<commit_message>
correccion logueo, y decodificacion de token
</commit_message>
<xml_diff>
--- a/uploads/CALCULADORA_V2.xlsx
+++ b/uploads/CALCULADORA_V2.xlsx
@@ -5009,7 +5009,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>10</v>
+        <v>60</v>
       </c>
       <c r="B3" t="str">
         <v>ALUMNOS DE CICLO I</v>
@@ -5849,7 +5849,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>180</v>
+        <v>70</v>
       </c>
       <c r="B3" t="str">
         <v>ALUMNOS TOTALES</v>
@@ -6737,7 +6737,7 @@
     </row>
     <row r="3">
       <c r="A3">
-        <v>150</v>
+        <v>50</v>
       </c>
       <c r="B3" t="str">
         <v>ALUMNOS TOTALES</v>

</xml_diff>